<commit_message>
Daily Orchestration - 2025-05-09
</commit_message>
<xml_diff>
--- a/reports/portfolio.xlsx
+++ b/reports/portfolio.xlsx
@@ -916,7 +916,7 @@
         <v>0.4</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.2975571955815117</v>
+        <v>0.2975571955815119</v>
       </c>
       <c r="BE2" t="n">
         <v>0.2509375164549231</v>
@@ -1105,16 +1105,16 @@
         <v>0.01</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.3444875939983535</v>
+        <v>0.3444875764013322</v>
       </c>
       <c r="BD3" t="n">
-        <v>0.3953672586989012</v>
+        <v>0.3953672586989023</v>
       </c>
       <c r="BE3" t="n">
         <v>0.3487884344335526</v>
       </c>
       <c r="BF3" t="n">
-        <v>1.133544635277241</v>
+        <v>1.133544635277244</v>
       </c>
     </row>
     <row r="4">
@@ -1297,16 +1297,16 @@
         <v>0.03</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.1487869805222688</v>
+        <v>0.1487869840215446</v>
       </c>
       <c r="BD4" t="n">
-        <v>0.1771429743888882</v>
+        <v>0.1771429743888884</v>
       </c>
       <c r="BE4" t="n">
         <v>0.2445850742488286</v>
       </c>
       <c r="BF4" t="n">
-        <v>0.7242591353251253</v>
+        <v>0.7242591353251263</v>
       </c>
     </row>
     <row r="5">
@@ -1489,16 +1489,16 @@
         <v>0.01</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.05672542547937767</v>
+        <v>0.05672543957712319</v>
       </c>
       <c r="BD5" t="n">
-        <v>0.1914359723221903</v>
+        <v>0.1914359723221908</v>
       </c>
       <c r="BE5" t="n">
         <v>0.2590738054284099</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.7389244621069574</v>
+        <v>0.7389244621069592</v>
       </c>
     </row>
     <row r="6">
@@ -1681,16 +1681,16 @@
         <v>0.01</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.05000000000000002</v>
+        <v>0.05</v>
       </c>
       <c r="BD6" t="n">
-        <v>0.1815321797512541</v>
+        <v>0.1815321797512546</v>
       </c>
       <c r="BE6" t="n">
         <v>0.2252337912391592</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.8059722244718533</v>
+        <v>0.8059722244718552</v>
       </c>
     </row>
   </sheetData>
@@ -40532,13 +40532,13 @@
         <v>0.1319</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.07745501207506189</v>
+        <v>-0.07745501207506178</v>
       </c>
       <c r="U5" t="n">
-        <v>0.1287197674737791</v>
+        <v>0.1287197674737792</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.9295775965368815</v>
+        <v>-0.9295775965368805</v>
       </c>
     </row>
     <row r="6">
@@ -40800,13 +40800,13 @@
         <v>0.1169</v>
       </c>
       <c r="T8" t="n">
-        <v>0.03715874556851584</v>
+        <v>0.03715874556851562</v>
       </c>
       <c r="U8" t="n">
-        <v>0.08846613923947173</v>
+        <v>0.08846613923947175</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.05698512984541835</v>
+        <v>-0.05698512984542085</v>
       </c>
     </row>
   </sheetData>
@@ -40880,19 +40880,19 @@
         <v>0.02183279542631911</v>
       </c>
       <c r="D2" t="n">
-        <v>1.134222798149796</v>
+        <v>1.134222798149797</v>
       </c>
       <c r="E2" t="n">
         <v>0.4449135172664331</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1979480378463884</v>
+        <v>0.1979480378463885</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0004145619378420125</v>
+        <v>0.0004145619378420083</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0690265924402271</v>
+        <v>0.06902659244022698</v>
       </c>
     </row>
     <row r="3">
@@ -40907,7 +40907,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.003068015869157018</v>
+        <v>0.003068015869157027</v>
       </c>
       <c r="D3" t="n">
         <v>1.349006020727707</v>
@@ -40919,10 +40919,10 @@
         <v>0.7085819427101692</v>
       </c>
       <c r="G3" t="n">
-        <v>6.802111858233947e-17</v>
+        <v>6.802111858234193e-17</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4947003706744052</v>
+        <v>0.4947003706744039</v>
       </c>
     </row>
     <row r="4">
@@ -40937,22 +40937,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0150516375337045</v>
+        <v>0.01505163753370451</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8324230809154241</v>
+        <v>0.8324230809154244</v>
       </c>
       <c r="E4" t="n">
         <v>0.5155511003422956</v>
       </c>
       <c r="F4" t="n">
-        <v>0.265792937064152</v>
+        <v>0.2657929370641516</v>
       </c>
       <c r="G4" t="n">
         <v>2.932419832694608e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>0.03940586626719852</v>
+        <v>0.03940586626719846</v>
       </c>
     </row>
     <row r="5">
@@ -40967,22 +40967,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.007755442603330645</v>
+        <v>0.00775544260333065</v>
       </c>
       <c r="D5" t="n">
         <v>1.015704665589921</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6176805693072802</v>
+        <v>0.6176805693072804</v>
       </c>
       <c r="F5" t="n">
         <v>0.3815292856997659</v>
       </c>
       <c r="G5" t="n">
-        <v>1.873698839416621e-07</v>
+        <v>1.873698839416607e-07</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2499880381859534</v>
+        <v>0.2499880381859533</v>
       </c>
     </row>
     <row r="6">
@@ -40997,22 +40997,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.006133821950291005</v>
+        <v>0.006133821950291007</v>
       </c>
       <c r="D6" t="n">
-        <v>0.982459637239831</v>
+        <v>0.9824596372398318</v>
       </c>
       <c r="E6" t="n">
-        <v>0.604007366477075</v>
+        <v>0.6040073664770751</v>
       </c>
       <c r="F6" t="n">
         <v>0.3648248987585714</v>
       </c>
       <c r="G6" t="n">
-        <v>4.08797392024918e-07</v>
+        <v>4.087973920249121e-07</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3630187857337297</v>
+        <v>0.3630187857337296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily Orchestration - 2025-05-10
</commit_message>
<xml_diff>
--- a/reports/portfolio.xlsx
+++ b/reports/portfolio.xlsx
@@ -40233,7 +40233,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>46887535579</v>
+        <v>47129940736</v>
       </c>
       <c r="L2" t="n">
         <v>239454</v>
@@ -40323,7 +40323,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>599087514</v>
+        <v>599704097</v>
       </c>
       <c r="L3" t="n">
         <v>239424</v>
@@ -40413,7 +40413,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2466639696</v>
+        <v>2474365039</v>
       </c>
       <c r="L4" t="n">
         <v>239423</v>
@@ -40503,7 +40503,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>9956934118</v>
+        <v>9952338249</v>
       </c>
       <c r="L5" t="n">
         <v>239453</v>
@@ -40593,7 +40593,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>981851249</v>
+        <v>992955881</v>
       </c>
       <c r="L6" t="n">
         <v>239830</v>
@@ -40683,7 +40683,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>28793916886</v>
+        <v>29316619618</v>
       </c>
       <c r="L7" t="n">
         <v>239566</v>
@@ -40771,7 +40771,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>89760939</v>
+        <v>89759396</v>
       </c>
       <c r="L8" t="n">
         <v>294319</v>

</xml_diff>

<commit_message>
Major Update: Dashboard, Pipeline, Orchestrator
</commit_message>
<xml_diff>
--- a/reports/portfolio.xlsx
+++ b/reports/portfolio.xlsx
@@ -741,7 +741,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -770,10 +770,10 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>166288293888</v>
+        <v>166786596864</v>
       </c>
       <c r="I2" t="n">
-        <v>170392190976</v>
+        <v>170544611328</v>
       </c>
       <c r="J2" t="n">
         <v>584007718</v>
@@ -782,19 +782,19 @@
         <v>586224000</v>
       </c>
       <c r="L2" t="n">
-        <v>19.11</v>
+        <v>19.18</v>
       </c>
       <c r="M2" t="n">
-        <v>20.56</v>
+        <v>20.62</v>
       </c>
       <c r="N2" t="n">
         <v>2.12</v>
       </c>
       <c r="O2" t="n">
-        <v>5.74</v>
+        <v>5.76</v>
       </c>
       <c r="P2" t="n">
-        <v>14.72</v>
+        <v>14.74</v>
       </c>
       <c r="Q2" t="n">
         <v>2.17</v>
@@ -824,7 +824,7 @@
         <v>0.184</v>
       </c>
       <c r="Z2" t="n">
-        <v>14.84</v>
+        <v>14.83</v>
       </c>
       <c r="AA2" t="n">
         <v>13.8</v>
@@ -860,7 +860,7 @@
         <v>16026999808</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.0173</v>
+        <v>0.0171</v>
       </c>
       <c r="AM2" t="n">
         <v>0.049</v>
@@ -872,7 +872,7 @@
         <v>0.3304</v>
       </c>
       <c r="AP2" t="n">
-        <v>283.66</v>
+        <v>284.51</v>
       </c>
       <c r="AQ2" t="n">
         <v>293.88</v>
@@ -901,10 +901,10 @@
         <v>201.34</v>
       </c>
       <c r="AY2" t="n">
-        <v>275.69</v>
+        <v>275.85</v>
       </c>
       <c r="AZ2" t="n">
-        <v>253.64</v>
+        <v>253.97</v>
       </c>
       <c r="BA2" t="n">
         <v>1.54</v>
@@ -933,7 +933,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -962,10 +962,10 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>222448959488</v>
+        <v>229231198208</v>
       </c>
       <c r="I3" t="n">
-        <v>230374260736</v>
+        <v>236655263744</v>
       </c>
       <c r="J3" t="n">
         <v>1062600970</v>
@@ -974,22 +974,22 @@
         <v>1066390016</v>
       </c>
       <c r="L3" t="n">
-        <v>32.9</v>
+        <v>33.91</v>
       </c>
       <c r="M3" t="n">
-        <v>39.81</v>
+        <v>41.02</v>
       </c>
       <c r="N3" t="n">
-        <v>5.61</v>
+        <v>5.78</v>
       </c>
       <c r="O3" t="n">
-        <v>11.55</v>
+        <v>11.91</v>
       </c>
       <c r="P3" t="n">
-        <v>23.6</v>
+        <v>24.24</v>
       </c>
       <c r="Q3" t="n">
-        <v>5.81</v>
+        <v>5.96</v>
       </c>
       <c r="R3" t="n">
         <v>0.3188</v>
@@ -1064,7 +1064,7 @@
         <v>0.2334</v>
       </c>
       <c r="AP3" t="n">
-        <v>208.6</v>
+        <v>214.96</v>
       </c>
       <c r="AQ3" t="n">
         <v>223.74</v>
@@ -1087,16 +1087,16 @@
         <v>1.31</v>
       </c>
       <c r="AW3" t="n">
-        <v>214.21</v>
+        <v>216.12</v>
       </c>
       <c r="AX3" t="n">
         <v>150.2</v>
       </c>
       <c r="AY3" t="n">
-        <v>195.86</v>
+        <v>196.08</v>
       </c>
       <c r="AZ3" t="n">
-        <v>183.72</v>
+        <v>183.97</v>
       </c>
       <c r="BA3" t="n">
         <v>1.67</v>
@@ -1105,7 +1105,7 @@
         <v>0.01</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.347636304435301</v>
+        <v>0.3476363140104058</v>
       </c>
       <c r="BD3" t="n">
         <v>0.3956092792739951</v>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1154,34 +1154,34 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>288177225728</v>
+        <v>276834058240</v>
       </c>
       <c r="I4" t="n">
-        <v>397864960000</v>
+        <v>386521858048</v>
       </c>
       <c r="J4" t="n">
-        <v>452156951</v>
+        <v>452134242</v>
       </c>
       <c r="K4" t="n">
         <v>1135449984</v>
       </c>
       <c r="L4" t="n">
-        <v>24.81</v>
+        <v>23.79</v>
       </c>
       <c r="M4" t="n">
-        <v>23.79</v>
+        <v>22.85</v>
       </c>
       <c r="N4" t="n">
-        <v>3.48</v>
+        <v>3.35</v>
       </c>
       <c r="O4" t="n">
-        <v>4.72</v>
+        <v>4.54</v>
       </c>
       <c r="P4" t="n">
-        <v>12.59</v>
+        <v>12.23</v>
       </c>
       <c r="Q4" t="n">
-        <v>4.81</v>
+        <v>4.67</v>
       </c>
       <c r="R4" t="n">
         <v>0.6385</v>
@@ -1208,7 +1208,7 @@
         <v>0.066</v>
       </c>
       <c r="Z4" t="n">
-        <v>10.23</v>
+        <v>10.24</v>
       </c>
       <c r="AA4" t="n">
         <v>10.67</v>
@@ -1244,7 +1244,7 @@
         <v>24056000512</v>
       </c>
       <c r="AL4" t="n">
-        <v>0.0139</v>
+        <v>0.014</v>
       </c>
       <c r="AM4" t="n">
         <v>0.0352</v>
@@ -1256,10 +1256,10 @@
         <v>0.2988</v>
       </c>
       <c r="AP4" t="n">
-        <v>253.8</v>
+        <v>243.81</v>
       </c>
       <c r="AQ4" t="n">
-        <v>269.25</v>
+        <v>269.57</v>
       </c>
       <c r="AR4" t="n">
         <v>305</v>
@@ -1285,19 +1285,19 @@
         <v>161.72</v>
       </c>
       <c r="AY4" t="n">
-        <v>258.31</v>
+        <v>257.93</v>
       </c>
       <c r="AZ4" t="n">
-        <v>228.02</v>
+        <v>228.37</v>
       </c>
       <c r="BA4" t="n">
-        <v>2.71</v>
+        <v>2.29</v>
       </c>
       <c r="BB4" t="n">
         <v>0.03</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.1423085131681223</v>
+        <v>0.1423085216298818</v>
       </c>
       <c r="BD4" t="n">
         <v>0.1734310432895125</v>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1346,10 +1346,10 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>143424307200</v>
+        <v>143022374912</v>
       </c>
       <c r="I5" t="n">
-        <v>150945726464</v>
+        <v>150543564800</v>
       </c>
       <c r="J5" t="n">
         <v>1114419446</v>
@@ -1358,22 +1358,22 @@
         <v>1116489984</v>
       </c>
       <c r="L5" t="n">
-        <v>30.15</v>
+        <v>30.07</v>
       </c>
       <c r="M5" t="n">
-        <v>27.93</v>
+        <v>27.85</v>
       </c>
       <c r="N5" t="n">
         <v>2.54</v>
       </c>
       <c r="O5" t="n">
-        <v>17.13</v>
+        <v>17.08</v>
       </c>
       <c r="P5" t="n">
-        <v>20.38</v>
+        <v>20.33</v>
       </c>
       <c r="Q5" t="n">
-        <v>2.68</v>
+        <v>2.67</v>
       </c>
       <c r="R5" t="n">
         <v>0.306</v>
@@ -1400,7 +1400,7 @@
         <v>-0.004</v>
       </c>
       <c r="Z5" t="n">
-        <v>4.26</v>
+        <v>4.27</v>
       </c>
       <c r="AA5" t="n">
         <v>4.6</v>
@@ -1448,7 +1448,7 @@
         <v>0.3421</v>
       </c>
       <c r="AP5" t="n">
-        <v>128.46</v>
+        <v>128.1</v>
       </c>
       <c r="AQ5" t="n">
         <v>134.43</v>
@@ -1474,22 +1474,22 @@
         <v>131.3</v>
       </c>
       <c r="AX5" t="n">
-        <v>97.47</v>
+        <v>97.53</v>
       </c>
       <c r="AY5" t="n">
-        <v>122.69</v>
+        <v>122.81</v>
       </c>
       <c r="AZ5" t="n">
-        <v>119.76</v>
+        <v>119.85</v>
       </c>
       <c r="BA5" t="n">
-        <v>2.07</v>
+        <v>2.14</v>
       </c>
       <c r="BB5" t="n">
         <v>0.01</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.06005518239657655</v>
+        <v>0.06005516435971234</v>
       </c>
       <c r="BD5" t="n">
         <v>0.1912884870395601</v>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1538,10 +1538,10 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>210437160960</v>
+        <v>213077934080</v>
       </c>
       <c r="I6" t="n">
-        <v>230726074368</v>
+        <v>233370042368</v>
       </c>
       <c r="J6" t="n">
         <v>469592833</v>
@@ -1550,22 +1550,22 @@
         <v>470724000</v>
       </c>
       <c r="L6" t="n">
-        <v>32.47</v>
+        <v>32.9</v>
       </c>
       <c r="M6" t="n">
-        <v>26.37</v>
+        <v>26.71</v>
       </c>
       <c r="N6" t="n">
-        <v>6.37</v>
+        <v>6.45</v>
       </c>
       <c r="O6" t="n">
-        <v>5.54</v>
+        <v>5.61</v>
       </c>
       <c r="P6" t="n">
-        <v>17.99</v>
+        <v>18.2</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.99</v>
+        <v>7.07</v>
       </c>
       <c r="R6" t="n">
         <v>0.4826</v>
@@ -1592,7 +1592,7 @@
         <v>0.001</v>
       </c>
       <c r="Z6" t="n">
-        <v>13.77</v>
+        <v>13.76</v>
       </c>
       <c r="AA6" t="n">
         <v>16.95</v>
@@ -1628,7 +1628,7 @@
         <v>9630000128</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.0134</v>
+        <v>0.0133</v>
       </c>
       <c r="AM6" t="n">
         <v>0.06</v>
@@ -1640,7 +1640,7 @@
         <v>0.4115</v>
       </c>
       <c r="AP6" t="n">
-        <v>447.05</v>
+        <v>452.66</v>
       </c>
       <c r="AQ6" t="n">
         <v>491.33</v>
@@ -1669,13 +1669,13 @@
         <v>408.65</v>
       </c>
       <c r="AY6" t="n">
-        <v>454.41</v>
+        <v>454.05</v>
       </c>
       <c r="AZ6" t="n">
-        <v>454.46</v>
+        <v>454.49</v>
       </c>
       <c r="BA6" t="n">
-        <v>1.81</v>
+        <v>1.99</v>
       </c>
       <c r="BB6" t="n">
         <v>0.01</v>
@@ -1684,13 +1684,13 @@
         <v>0.05</v>
       </c>
       <c r="BD6" t="n">
-        <v>0.1810768354019361</v>
+        <v>0.1810768354019359</v>
       </c>
       <c r="BE6" t="n">
         <v>0.2251458589893061</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.8042645608264855</v>
+        <v>0.8042645608264845</v>
       </c>
     </row>
   </sheetData>
@@ -1767,9 +1767,7 @@
       <c r="H2" t="n">
         <v>142.63</v>
       </c>
-      <c r="I2" t="n">
-        <v>30.26</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -1784,9 +1782,7 @@
       <c r="H3" t="n">
         <v>145.02</v>
       </c>
-      <c r="I3" t="n">
-        <v>30.74</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -1801,9 +1797,7 @@
       <c r="H4" t="n">
         <v>143.13</v>
       </c>
-      <c r="I4" t="n">
-        <v>31.25</v>
-      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -38167,7 +38161,9 @@
       <c r="H1258" t="n">
         <v>87.53</v>
       </c>
-      <c r="I1258" t="inlineStr"/>
+      <c r="I1258" t="n">
+        <v>55.01</v>
+      </c>
     </row>
     <row r="1259">
       <c r="A1259" s="3" t="n">
@@ -38223,7 +38219,9 @@
       <c r="H1260" t="n">
         <v>86.94</v>
       </c>
-      <c r="I1260" t="inlineStr"/>
+      <c r="I1260" t="n">
+        <v>55.03</v>
+      </c>
     </row>
     <row r="1261">
       <c r="A1261" s="3" t="n">
@@ -40285,19 +40283,19 @@
         <v>0.029</v>
       </c>
       <c r="R2" t="n">
-        <v>18.131</v>
+        <v>18.136</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1813</v>
+        <v>0.1814</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.1060335059639883</v>
+        <v>-0.1054461676013334</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1626933704392784</v>
+        <v>0.1625784504382385</v>
       </c>
       <c r="V2" t="n">
-        <v>-0.9111219809618063</v>
+        <v>-0.9081533696707385</v>
       </c>
     </row>
     <row r="3">
@@ -40366,7 +40364,7 @@
         <v>0.056</v>
       </c>
       <c r="O3" t="n">
-        <v>21.92</v>
+        <v>21.91</v>
       </c>
       <c r="P3" t="n">
         <v>2.35</v>
@@ -40375,19 +40373,19 @@
         <v>0.04</v>
       </c>
       <c r="R3" t="n">
-        <v>14.881</v>
+        <v>14.884</v>
       </c>
       <c r="S3" t="n">
         <v>0.1488</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.04636964646664399</v>
+        <v>-0.0449504312791581</v>
       </c>
       <c r="U3" t="n">
-        <v>0.1281544189006788</v>
+        <v>0.1281565144316112</v>
       </c>
       <c r="V3" t="n">
-        <v>-0.6911166015686629</v>
+        <v>-0.6800312232716392</v>
       </c>
     </row>
     <row r="4">
@@ -40456,7 +40454,7 @@
         <v>0.06</v>
       </c>
       <c r="O4" t="n">
-        <v>22.13</v>
+        <v>22.14</v>
       </c>
       <c r="P4" t="n">
         <v>2.17</v>
@@ -40465,19 +40463,19 @@
         <v>0.046</v>
       </c>
       <c r="R4" t="n">
-        <v>14.583</v>
+        <v>14.58</v>
       </c>
       <c r="S4" t="n">
         <v>0.1458</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.02621458185552727</v>
+        <v>-0.02265030981166838</v>
       </c>
       <c r="U4" t="n">
-        <v>0.1270233075687072</v>
+        <v>0.127019833245691</v>
       </c>
       <c r="V4" t="n">
-        <v>-0.5385986490591235</v>
+        <v>-0.5105526291018677</v>
       </c>
     </row>
     <row r="5">
@@ -40555,19 +40553,19 @@
         <v>0.032</v>
       </c>
       <c r="R5" t="n">
-        <v>13.185</v>
+        <v>13.187</v>
       </c>
       <c r="S5" t="n">
         <v>0.1319</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.07710092205691832</v>
+        <v>-0.07678980925276147</v>
       </c>
       <c r="U5" t="n">
-        <v>0.1286713622100245</v>
+        <v>0.1286332756246679</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.9271754025747293</v>
+        <v>-0.9250313239317285</v>
       </c>
     </row>
     <row r="6">
@@ -40636,7 +40634,7 @@
         <v>0.028</v>
       </c>
       <c r="O6" t="n">
-        <v>9.640000000000001</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P6" t="n">
         <v>1.12</v>
@@ -40645,19 +40643,19 @@
         <v>0.022</v>
       </c>
       <c r="R6" t="n">
-        <v>8.535</v>
+        <v>8.534000000000001</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0854</v>
+        <v>0.0853</v>
       </c>
       <c r="T6" t="n">
-        <v>-0.03683784735637596</v>
+        <v>-0.03636568790852834</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0955614452753703</v>
+        <v>0.09564284653000403</v>
       </c>
       <c r="V6" t="n">
-        <v>-0.8270892840582321</v>
+        <v>-0.8214486577820701</v>
       </c>
     </row>
     <row r="7">
@@ -40741,13 +40739,13 @@
         <v>0.0974</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.005158556261155689</v>
+        <v>-0.00298836392802504</v>
       </c>
       <c r="U7" t="n">
-        <v>0.08791887439810174</v>
+        <v>0.08790196789783455</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.5386619947693303</v>
+        <v>-0.5140768177175046</v>
       </c>
     </row>
     <row r="8">
@@ -40829,13 +40827,13 @@
         <v>0.1169</v>
       </c>
       <c r="T8" t="n">
-        <v>0.03680488612450605</v>
+        <v>0.03860478720909666</v>
       </c>
       <c r="U8" t="n">
-        <v>0.08843431556151986</v>
+        <v>0.08835072958674264</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.06100701793457991</v>
+        <v>-0.04069250823077313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>